<commit_message>
Fix Semi toujours 30t + fallback POILOUR + ACHREF SEMI uniquement
</commit_message>
<xml_diff>
--- a/transport_etat_final.xlsx
+++ b/transport_etat_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amset\Desktop\Tomate_scheduler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B357C9-DAFF-432D-911A-C233C0FC1CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29C9C65-2758-464C-B7E0-C4EA214AC5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="11340" windowHeight="10848" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="liste confirmé" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="277">
   <si>
     <t>Longueur  de caisse</t>
   </si>
@@ -789,9 +789,6 @@
   </si>
   <si>
     <t>Morad Ghali</t>
-  </si>
-  <si>
-    <t>Semi Double Rem</t>
   </si>
   <si>
     <t>El Mida</t>
@@ -2774,7 +2771,7 @@
         <v>239</v>
       </c>
       <c r="E34" s="24" t="s">
-        <v>19</v>
+        <v>261</v>
       </c>
       <c r="F34" s="14" t="s">
         <v>139</v>
@@ -3648,7 +3645,7 @@
         <v>62</v>
       </c>
       <c r="E59" s="19" t="s">
-        <v>251</v>
+        <v>104</v>
       </c>
       <c r="F59" s="8" t="s">
         <v>61</v>
@@ -4333,7 +4330,7 @@
         <v>73</v>
       </c>
       <c r="B78" s="22">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C78" s="48">
         <v>6</v>
@@ -5605,10 +5602,10 @@
         <v>70</v>
       </c>
       <c r="F113" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G113" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H113" s="24"/>
       <c r="I113" s="14" t="s">
@@ -5691,16 +5688,16 @@
         <v>248</v>
       </c>
       <c r="D116" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E116" s="14" t="s">
         <v>70</v>
       </c>
       <c r="F116" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G116" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H116" s="14">
         <v>97258836</v>
@@ -5731,7 +5728,7 @@
         <v>19</v>
       </c>
       <c r="F117" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G117" s="14" t="s">
         <v>122</v>
@@ -5765,7 +5762,7 @@
         <v>19</v>
       </c>
       <c r="F118" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G118" s="14" t="s">
         <v>122</v>
@@ -5799,10 +5796,10 @@
         <v>19</v>
       </c>
       <c r="F119" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="G119" s="14" t="s">
         <v>264</v>
-      </c>
-      <c r="G119" s="14" t="s">
-        <v>265</v>
       </c>
       <c r="H119" s="14">
         <v>21318143</v>
@@ -5835,7 +5832,7 @@
         <v>19</v>
       </c>
       <c r="F120" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G120" s="14" t="s">
         <v>122</v>
@@ -5865,10 +5862,10 @@
         <v>19</v>
       </c>
       <c r="F121" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G121" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H121" s="14"/>
       <c r="I121" s="14" t="s">
@@ -5897,7 +5894,7 @@
         <v>19</v>
       </c>
       <c r="F122" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G122" s="14" t="s">
         <v>110</v>
@@ -5927,10 +5924,10 @@
         <v>70</v>
       </c>
       <c r="F123" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="G123" s="14" t="s">
         <v>258</v>
-      </c>
-      <c r="G123" s="14" t="s">
-        <v>259</v>
       </c>
       <c r="H123" s="14">
         <v>54379394</v>
@@ -5957,10 +5954,10 @@
         <v>19</v>
       </c>
       <c r="F124" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G124" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H124" s="14">
         <v>21153960</v>
@@ -5982,13 +5979,13 @@
       </c>
       <c r="D125" s="14"/>
       <c r="E125" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F125" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G125" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H125" s="14">
         <v>21153960</v>
@@ -6013,7 +6010,7 @@
         <v>19</v>
       </c>
       <c r="F126" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G126" s="14" t="s">
         <v>125</v>
@@ -6041,7 +6038,7 @@
         <v>68</v>
       </c>
       <c r="F127" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G127" s="14" t="s">
         <v>113</v>
@@ -6073,7 +6070,7 @@
         <v>68</v>
       </c>
       <c r="F128" s="14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G128" s="14" t="s">
         <v>124</v>
@@ -6109,7 +6106,7 @@
         <v>68</v>
       </c>
       <c r="F129" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G129" s="14" t="s">
         <v>124</v>
@@ -6139,13 +6136,13 @@
         <v>6</v>
       </c>
       <c r="D130" s="14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E130" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F130" s="14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G130" s="14" t="s">
         <v>113</v>
@@ -6177,16 +6174,16 @@
         <v>6</v>
       </c>
       <c r="D131" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E131" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F131" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G131" s="14" t="s">
         <v>267</v>
-      </c>
-      <c r="G131" s="14" t="s">
-        <v>268</v>
       </c>
       <c r="H131" s="14">
         <v>22060453</v>
@@ -6215,16 +6212,16 @@
         <v>6</v>
       </c>
       <c r="D132" s="14" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E132" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F132" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="G132" s="14" t="s">
         <v>269</v>
-      </c>
-      <c r="G132" s="14" t="s">
-        <v>270</v>
       </c>
       <c r="H132" s="14">
         <v>50433962</v>
@@ -6248,7 +6245,7 @@
       </c>
       <c r="B133" s="50">
         <f>SUM(B2:B132)</f>
-        <v>2464</v>
+        <v>2449</v>
       </c>
       <c r="C133" s="14"/>
       <c r="D133" s="14"/>

</xml_diff>

<commit_message>
Fix: overflow ELFALLEH x2000, arrondi 5t, onglet comparaison plans OR-Tools vs Manuel
</commit_message>
<xml_diff>
--- a/transport_etat_final.xlsx
+++ b/transport_etat_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amset\Desktop\Tomate_scheduler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29C9C65-2758-464C-B7E0-C4EA214AC5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9130B3F-7F11-4530-A9F9-304786A17C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1518,6 +1518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L3466"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1575,7 +1576,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>73</v>
       </c>
@@ -1613,7 +1614,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>202</v>
       </c>
@@ -1689,7 +1690,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>73</v>
       </c>
@@ -1727,7 +1728,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>73</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>73</v>
       </c>
@@ -1803,7 +1804,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>73</v>
       </c>
@@ -1841,7 +1842,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
         <v>73</v>
       </c>
@@ -1877,7 +1878,7 @@
       </c>
       <c r="L9" s="22"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
         <v>73</v>
       </c>
@@ -1915,7 +1916,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>134</v>
       </c>
@@ -1949,7 +1950,7 @@
       <c r="K11" s="14"/>
       <c r="L11" s="22"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>73</v>
       </c>
@@ -1983,7 +1984,7 @@
       <c r="K12" s="14"/>
       <c r="L12" s="22"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>73</v>
       </c>
@@ -2021,7 +2022,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
         <v>73</v>
       </c>
@@ -2057,7 +2058,7 @@
       </c>
       <c r="L14" s="22"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
         <v>75</v>
       </c>
@@ -2091,7 +2092,7 @@
       </c>
       <c r="L15" s="22"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
         <v>133</v>
       </c>
@@ -2125,7 +2126,7 @@
       <c r="K16" s="14"/>
       <c r="L16" s="22"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>74</v>
       </c>
@@ -2163,7 +2164,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
         <v>74</v>
       </c>
@@ -2201,7 +2202,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
         <v>73</v>
       </c>
@@ -2239,7 +2240,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
         <v>73</v>
       </c>
@@ -2275,7 +2276,7 @@
       </c>
       <c r="L20" s="22"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
         <v>134</v>
       </c>
@@ -2313,7 +2314,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
         <v>74</v>
       </c>
@@ -2349,7 +2350,7 @@
       </c>
       <c r="L22" s="22"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
         <v>74</v>
       </c>
@@ -2387,7 +2388,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
         <v>73</v>
       </c>
@@ -2423,7 +2424,7 @@
       </c>
       <c r="L24" s="22"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>73</v>
       </c>
@@ -2459,7 +2460,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
         <v>73</v>
       </c>
@@ -2497,7 +2498,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>134</v>
       </c>
@@ -2533,7 +2534,7 @@
       </c>
       <c r="L27" s="22"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
         <v>73</v>
       </c>
@@ -2571,7 +2572,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
         <v>73</v>
       </c>
@@ -2609,7 +2610,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
         <v>73</v>
       </c>
@@ -2683,7 +2684,7 @@
       </c>
       <c r="L31" s="22"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
         <v>73</v>
       </c>
@@ -2863,7 +2864,7 @@
       </c>
       <c r="L36" s="22"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
         <v>73</v>
       </c>
@@ -2897,7 +2898,7 @@
       <c r="K37" s="14"/>
       <c r="L37" s="22"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
         <v>73</v>
       </c>
@@ -2931,7 +2932,7 @@
       <c r="K38" s="14"/>
       <c r="L38" s="22"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
         <v>73</v>
       </c>
@@ -2959,7 +2960,7 @@
       <c r="K39" s="14"/>
       <c r="L39" s="22"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="14" t="s">
         <v>73</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>73</v>
       </c>
@@ -3011,7 +3012,7 @@
         <v>31</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>32</v>
@@ -3035,7 +3036,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
         <v>73</v>
       </c>
@@ -3073,7 +3074,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>73</v>
       </c>
@@ -3141,7 +3142,7 @@
       <c r="K44" s="14"/>
       <c r="L44" s="22"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>74</v>
       </c>
@@ -3173,7 +3174,7 @@
       <c r="K45" s="14"/>
       <c r="L45" s="22"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
         <v>73</v>
       </c>
@@ -3211,7 +3212,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
         <v>74</v>
       </c>
@@ -3249,7 +3250,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
         <v>74</v>
       </c>
@@ -3281,7 +3282,7 @@
       <c r="K48" s="14"/>
       <c r="L48" s="22"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="14" t="s">
         <v>73</v>
       </c>
@@ -3315,7 +3316,7 @@
       <c r="K49" s="14"/>
       <c r="L49" s="22"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
         <v>73</v>
       </c>
@@ -3353,7 +3354,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="14" t="s">
         <v>74</v>
       </c>
@@ -3389,7 +3390,7 @@
       </c>
       <c r="L51" s="22"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="14" t="s">
         <v>73</v>
       </c>
@@ -3425,7 +3426,7 @@
       </c>
       <c r="L52" s="22"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
         <v>73</v>
       </c>
@@ -3461,7 +3462,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="14" t="s">
         <v>74</v>
       </c>
@@ -3495,7 +3496,7 @@
       <c r="K54" s="14"/>
       <c r="L54" s="22"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="14" t="s">
         <v>74</v>
       </c>
@@ -3529,7 +3530,7 @@
       <c r="K55" s="14"/>
       <c r="L55" s="22"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="14" t="s">
         <v>74</v>
       </c>
@@ -3563,7 +3564,7 @@
       <c r="K56" s="14"/>
       <c r="L56" s="22"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="14" t="s">
         <v>74</v>
       </c>
@@ -3597,7 +3598,7 @@
       <c r="K57" s="14"/>
       <c r="L57" s="22"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="14" t="s">
         <v>75</v>
       </c>
@@ -3631,7 +3632,7 @@
       <c r="K58" s="14"/>
       <c r="L58" s="22"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="14" t="s">
         <v>75</v>
       </c>
@@ -3665,7 +3666,7 @@
       <c r="K59" s="14"/>
       <c r="L59" s="22"/>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="14" t="s">
         <v>75</v>
       </c>
@@ -3697,7 +3698,7 @@
       <c r="K60" s="14"/>
       <c r="L60" s="22"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="14" t="s">
         <v>154</v>
       </c>
@@ -3729,7 +3730,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="14" t="s">
         <v>74</v>
       </c>
@@ -3767,7 +3768,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="14" t="s">
         <v>73</v>
       </c>
@@ -3805,7 +3806,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="14" t="s">
         <v>75</v>
       </c>
@@ -3841,7 +3842,7 @@
       </c>
       <c r="L64" s="22"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="14" t="s">
         <v>75</v>
       </c>
@@ -3915,7 +3916,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="14" t="s">
         <v>73</v>
       </c>
@@ -3953,7 +3954,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="14" t="s">
         <v>73</v>
       </c>
@@ -3989,7 +3990,7 @@
       </c>
       <c r="L68" s="22"/>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="14" t="s">
         <v>73</v>
       </c>
@@ -4025,7 +4026,7 @@
       </c>
       <c r="L69" s="22"/>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="14" t="s">
         <v>73</v>
       </c>
@@ -4063,7 +4064,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="14" t="s">
         <v>203</v>
       </c>
@@ -4101,7 +4102,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="14" t="s">
         <v>73</v>
       </c>
@@ -4139,7 +4140,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="14" t="s">
         <v>73</v>
       </c>
@@ -4177,7 +4178,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="14" t="s">
         <v>73</v>
       </c>
@@ -4215,7 +4216,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="14" t="s">
         <v>74</v>
       </c>
@@ -4253,7 +4254,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="14" t="s">
         <v>74</v>
       </c>
@@ -4325,7 +4326,7 @@
       </c>
       <c r="L77" s="22"/>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="14" t="s">
         <v>73</v>
       </c>
@@ -4399,7 +4400,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="14" t="s">
         <v>73</v>
       </c>
@@ -4437,7 +4438,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="14" t="s">
         <v>75</v>
       </c>
@@ -4473,7 +4474,7 @@
       </c>
       <c r="L81" s="22"/>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="14" t="s">
         <v>75</v>
       </c>
@@ -4509,7 +4510,7 @@
       </c>
       <c r="L82" s="22"/>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="14" t="s">
         <v>73</v>
       </c>
@@ -4541,7 +4542,7 @@
       <c r="K83" s="14"/>
       <c r="L83" s="22"/>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="14" t="s">
         <v>73</v>
       </c>
@@ -4611,7 +4612,7 @@
       </c>
       <c r="L85" s="22"/>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="14" t="s">
         <v>74</v>
       </c>
@@ -4649,7 +4650,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="14" t="s">
         <v>88</v>
       </c>
@@ -4687,7 +4688,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="14" t="s">
         <v>88</v>
       </c>
@@ -4723,7 +4724,7 @@
       </c>
       <c r="L88" s="22"/>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="14" t="s">
         <v>103</v>
       </c>
@@ -4755,7 +4756,7 @@
       <c r="K89" s="14"/>
       <c r="L89" s="22"/>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="14" t="s">
         <v>103</v>
       </c>
@@ -4793,7 +4794,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="14" t="s">
         <v>74</v>
       </c>
@@ -4831,7 +4832,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="14" t="s">
         <v>73</v>
       </c>
@@ -4845,7 +4846,7 @@
         <v>207</v>
       </c>
       <c r="E92" s="14" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="F92" s="14" t="s">
         <v>161</v>
@@ -4869,7 +4870,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="14" t="s">
         <v>133</v>
       </c>
@@ -4903,7 +4904,7 @@
       <c r="K93" s="14"/>
       <c r="L93" s="16"/>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="14" t="s">
         <v>133</v>
       </c>
@@ -4937,7 +4938,7 @@
       <c r="K94" s="14"/>
       <c r="L94" s="22"/>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="14" t="s">
         <v>73</v>
       </c>
@@ -4951,7 +4952,7 @@
         <v>208</v>
       </c>
       <c r="E95" s="14" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="F95" s="14" t="s">
         <v>161</v>
@@ -4973,7 +4974,7 @@
       </c>
       <c r="L95" s="22"/>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="14" t="s">
         <v>73</v>
       </c>
@@ -5011,7 +5012,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="14" t="s">
         <v>73</v>
       </c>
@@ -5049,7 +5050,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="14" t="s">
         <v>103</v>
       </c>
@@ -5085,7 +5086,7 @@
       </c>
       <c r="L98" s="22"/>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="14" t="s">
         <v>75</v>
       </c>
@@ -5121,7 +5122,7 @@
       </c>
       <c r="L99" s="22"/>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="14" t="s">
         <v>75</v>
       </c>
@@ -5159,7 +5160,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="14" t="s">
         <v>75</v>
       </c>
@@ -5195,7 +5196,7 @@
       </c>
       <c r="L101" s="22"/>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="14" t="s">
         <v>75</v>
       </c>
@@ -5233,7 +5234,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="14" t="s">
         <v>73</v>
       </c>
@@ -5269,7 +5270,7 @@
       </c>
       <c r="L103" s="22"/>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="14" t="s">
         <v>75</v>
       </c>
@@ -5307,7 +5308,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="14" t="s">
         <v>103</v>
       </c>
@@ -5343,7 +5344,7 @@
       </c>
       <c r="L105" s="22"/>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="14" t="s">
         <v>103</v>
       </c>
@@ -5381,7 +5382,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="14" t="s">
         <v>103</v>
       </c>
@@ -5417,7 +5418,7 @@
       </c>
       <c r="L107" s="22"/>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="14" t="s">
         <v>103</v>
       </c>
@@ -5453,7 +5454,7 @@
       </c>
       <c r="L108" s="22"/>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="14" t="s">
         <v>75</v>
       </c>
@@ -5489,7 +5490,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="14" t="s">
         <v>75</v>
       </c>
@@ -5523,7 +5524,7 @@
       <c r="K110" s="14"/>
       <c r="L110" s="22"/>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="14" t="s">
         <v>75</v>
       </c>
@@ -5555,7 +5556,7 @@
       <c r="K111" s="14"/>
       <c r="L111" s="22"/>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="14" t="s">
         <v>75</v>
       </c>
@@ -5649,7 +5650,7 @@
       <c r="K114" s="14"/>
       <c r="L114" s="22"/>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="14" t="s">
         <v>134</v>
       </c>
@@ -5713,7 +5714,7 @@
       </c>
       <c r="L116" s="14"/>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="14" t="s">
         <v>73</v>
       </c>
@@ -5747,7 +5748,7 @@
       </c>
       <c r="L117" s="14"/>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="14" t="s">
         <v>73</v>
       </c>
@@ -5781,7 +5782,7 @@
       </c>
       <c r="L118" s="14"/>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="14" t="s">
         <v>73</v>
       </c>
@@ -5817,7 +5818,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="14" t="s">
         <v>73</v>
       </c>
@@ -5847,7 +5848,7 @@
       <c r="K120" s="14"/>
       <c r="L120" s="14"/>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="14" t="s">
         <v>134</v>
       </c>
@@ -5879,7 +5880,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="14" t="s">
         <v>75</v>
       </c>
@@ -5909,7 +5910,7 @@
       <c r="K122" s="14"/>
       <c r="L122" s="14"/>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="14" t="s">
         <v>75</v>
       </c>
@@ -5939,7 +5940,7 @@
       <c r="K123" s="14"/>
       <c r="L123" s="14"/>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="14" t="s">
         <v>75</v>
       </c>
@@ -5967,7 +5968,7 @@
       <c r="K124" s="14"/>
       <c r="L124" s="14"/>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="14" t="s">
         <v>75</v>
       </c>
@@ -5995,7 +5996,7 @@
       <c r="K125" s="14"/>
       <c r="L125" s="14"/>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="14" t="s">
         <v>75</v>
       </c>
@@ -6023,7 +6024,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="14" t="s">
         <v>74</v>
       </c>
@@ -6055,7 +6056,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="14" t="s">
         <v>74</v>
       </c>
@@ -6091,7 +6092,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="14" t="s">
         <v>74</v>
       </c>
@@ -6125,7 +6126,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="14" t="s">
         <v>74</v>
       </c>
@@ -6163,7 +6164,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="14" t="s">
         <v>74</v>
       </c>
@@ -6201,7 +6202,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="14" t="s">
         <v>74</v>
       </c>
@@ -6239,7 +6240,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" ht="25.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="50" t="s">
         <v>249</v>
       </c>
@@ -6261,7 +6262,7 @@
         <v>221500</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="14"/>
       <c r="D134" s="1"/>
       <c r="H134" s="1"/>
@@ -19425,7 +19426,18 @@
       <c r="C3466" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L134" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L134" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Sicam"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Semi"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>